<commit_message>
Change classCode value from GRIC to GRICAWATIF ee3a3f0fdd4ae605aca65e2134e09478ac0a4647
</commit_message>
<xml_diff>
--- a/enrichissement-pharm/ig/StructureDefinition-FRCDAMaterialPharm.xlsx
+++ b/enrichissement-pharm/ig/StructureDefinition-FRCDAMaterialPharm.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-29T08:04:35+00:00</t>
+    <t>2026-07-29T08:58:09+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -582,7 +582,7 @@
     <t>Code indiquant qu'il s'agit d'une relation vers une classe générique ou thérapeutique.</t>
   </si>
   <si>
-    <t>GRIC</t>
+    <t>GRICAWATIF</t>
   </si>
   <si>
     <t>FRCDAMaterialPharm.asSpecializedKind.generalizedMedicineClass</t>

</xml_diff>

<commit_message>
Change classCode assignment to use hash syntax da043967627e252a83dcee0d6d5e75e59c8e9de3
</commit_message>
<xml_diff>
--- a/enrichissement-pharm/ig/StructureDefinition-FRCDAMaterialPharm.xlsx
+++ b/enrichissement-pharm/ig/StructureDefinition-FRCDAMaterialPharm.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-29T08:58:09+00:00</t>
+    <t>2026-07-29T09:37:21+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -582,7 +582,7 @@
     <t>Code indiquant qu'il s'agit d'une relation vers une classe générique ou thérapeutique.</t>
   </si>
   <si>
-    <t>GRICAWATIF</t>
+    <t>GRIC</t>
   </si>
   <si>
     <t>FRCDAMaterialPharm.asSpecializedKind.generalizedMedicineClass</t>

</xml_diff>